<commit_message>
princ markt mock up for pi AU and more
</commit_message>
<xml_diff>
--- a/stats for com eng/excel files/Ch06-02.xlsx
+++ b/stats for com eng/excel files/Ch06-02.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pin/Desktop/joint-repository/stats for com eng/excel files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB7FFBB-2B7E-C44A-A616-2DA13CD6A57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF00AFA1-DB29-DC4E-8E16-9D7AF94C61D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="24080" windowHeight="13180" activeTab="2" xr2:uid="{0900C177-0103-404A-B722-511C268DDC47}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="20480" windowHeight="11060" activeTab="1" xr2:uid="{0900C177-0103-404A-B722-511C268DDC47}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -443,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -533,18 +533,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7959,11 +7955,11 @@
         <v>0.44300299999999915</v>
       </c>
       <c r="K2" s="10">
-        <f>$J$26+$J$25*B2</f>
+        <f t="shared" ref="K2:K21" si="0">$J$26+$J$25*B2</f>
         <v>89.081319175185058</v>
       </c>
       <c r="L2" s="12">
-        <f t="shared" ref="L2:L21" si="0">C2-K2</f>
+        <f t="shared" ref="L2:L21" si="1">C2-K2</f>
         <v>0.92868082481494696</v>
       </c>
       <c r="M2" s="12">
@@ -7982,43 +7978,43 @@
         <v>89.05</v>
       </c>
       <c r="D3" s="4">
-        <f t="shared" ref="D3:D21" si="1">B3*C3</f>
+        <f t="shared" ref="D3:D21" si="2">B3*C3</f>
         <v>90.831000000000003</v>
       </c>
       <c r="E3" s="4">
-        <f t="shared" ref="E3:E21" si="2">B3*B3</f>
+        <f t="shared" ref="E3:E21" si="3">B3*B3</f>
         <v>1.0404</v>
       </c>
       <c r="F3" s="4">
-        <f t="shared" ref="F3:F20" si="3">C3*C3</f>
+        <f t="shared" ref="F3:F20" si="4">C3*C3</f>
         <v>7929.9024999999992</v>
       </c>
       <c r="G3" s="7">
-        <f>B3-B$23</f>
+        <f t="shared" ref="G3:G21" si="5">B3-B$23</f>
         <v>-0.17600000000000016</v>
       </c>
       <c r="H3" s="7">
-        <f t="shared" ref="H3:H21" si="4">C3-C$23</f>
+        <f t="shared" ref="H3:H21" si="6">C3-C$23</f>
         <v>-3.1105000000000018</v>
       </c>
       <c r="I3" s="8">
-        <f t="shared" ref="I3:I21" si="5">G3*G3</f>
+        <f t="shared" ref="I3:I21" si="7">G3*G3</f>
         <v>3.0976000000000056E-2</v>
       </c>
       <c r="J3" s="9">
-        <f t="shared" ref="J3:J21" si="6">G3*H3</f>
+        <f t="shared" ref="J3:J21" si="8">G3*H3</f>
         <v>0.54744800000000082</v>
       </c>
       <c r="K3" s="10">
-        <f>$J$26+$J$25*B3</f>
+        <f t="shared" si="0"/>
         <v>89.529743567148401</v>
       </c>
       <c r="L3" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.47974356714840383</v>
       </c>
       <c r="M3" s="12">
-        <f t="shared" ref="M3:M21" si="7">L3*L3</f>
+        <f t="shared" ref="M3:M21" si="9">L3*L3</f>
         <v>0.23015389022027505</v>
       </c>
     </row>
@@ -8033,43 +8029,43 @@
         <v>91.43</v>
       </c>
       <c r="D4" s="4">
+        <f t="shared" si="2"/>
+        <v>105.14449999999999</v>
+      </c>
+      <c r="E4" s="4">
+        <f t="shared" si="3"/>
+        <v>1.3224999999999998</v>
+      </c>
+      <c r="F4" s="4">
+        <f t="shared" si="4"/>
+        <v>8359.4449000000004</v>
+      </c>
+      <c r="G4" s="7">
+        <f t="shared" si="5"/>
+        <v>-4.6000000000000263E-2</v>
+      </c>
+      <c r="H4" s="7">
+        <f t="shared" si="6"/>
+        <v>-0.73049999999999216</v>
+      </c>
+      <c r="I4" s="8">
+        <f t="shared" si="7"/>
+        <v>2.1160000000000241E-3</v>
+      </c>
+      <c r="J4" s="9">
+        <f t="shared" si="8"/>
+        <v>3.3602999999999834E-2</v>
+      </c>
+      <c r="K4" s="10">
+        <f t="shared" si="0"/>
+        <v>91.472915932322877</v>
+      </c>
+      <c r="L4" s="12">
         <f t="shared" si="1"/>
-        <v>105.14449999999999</v>
-      </c>
-      <c r="E4" s="4">
-        <f t="shared" si="2"/>
-        <v>1.3224999999999998</v>
-      </c>
-      <c r="F4" s="4">
-        <f t="shared" si="3"/>
-        <v>8359.4449000000004</v>
-      </c>
-      <c r="G4" s="7">
-        <f>B4-B$23</f>
-        <v>-4.6000000000000263E-2</v>
-      </c>
-      <c r="H4" s="7">
-        <f t="shared" si="4"/>
-        <v>-0.73049999999999216</v>
-      </c>
-      <c r="I4" s="8">
-        <f t="shared" si="5"/>
-        <v>2.1160000000000241E-3</v>
-      </c>
-      <c r="J4" s="9">
-        <f t="shared" si="6"/>
-        <v>3.3602999999999834E-2</v>
-      </c>
-      <c r="K4" s="10">
-        <f>$J$26+$J$25*B4</f>
-        <v>91.472915932322877</v>
-      </c>
-      <c r="L4" s="12">
-        <f t="shared" si="0"/>
         <v>-4.2915932322870276E-2</v>
       </c>
       <c r="M4" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.8417772471411818E-3</v>
       </c>
     </row>
@@ -8084,43 +8080,43 @@
         <v>93.74</v>
       </c>
       <c r="D5" s="4">
+        <f t="shared" si="2"/>
+        <v>120.9246</v>
+      </c>
+      <c r="E5" s="4">
+        <f t="shared" si="3"/>
+        <v>1.6641000000000001</v>
+      </c>
+      <c r="F5" s="4">
+        <f t="shared" si="4"/>
+        <v>8787.1875999999993</v>
+      </c>
+      <c r="G5" s="7">
+        <f t="shared" si="5"/>
+        <v>9.3999999999999861E-2</v>
+      </c>
+      <c r="H5" s="7">
+        <f t="shared" si="6"/>
+        <v>1.5794999999999959</v>
+      </c>
+      <c r="I5" s="8">
+        <f t="shared" si="7"/>
+        <v>8.8359999999999741E-3</v>
+      </c>
+      <c r="J5" s="9">
+        <f t="shared" si="8"/>
+        <v>0.14847299999999938</v>
+      </c>
+      <c r="K5" s="10">
+        <f t="shared" si="0"/>
+        <v>93.565563094818472</v>
+      </c>
+      <c r="L5" s="12">
         <f t="shared" si="1"/>
-        <v>120.9246</v>
-      </c>
-      <c r="E5" s="4">
-        <f t="shared" si="2"/>
-        <v>1.6641000000000001</v>
-      </c>
-      <c r="F5" s="4">
-        <f t="shared" si="3"/>
-        <v>8787.1875999999993</v>
-      </c>
-      <c r="G5" s="7">
-        <f>B5-B$23</f>
-        <v>9.3999999999999861E-2</v>
-      </c>
-      <c r="H5" s="7">
-        <f t="shared" si="4"/>
-        <v>1.5794999999999959</v>
-      </c>
-      <c r="I5" s="8">
-        <f t="shared" si="5"/>
-        <v>8.8359999999999741E-3</v>
-      </c>
-      <c r="J5" s="9">
-        <f t="shared" si="6"/>
-        <v>0.14847299999999938</v>
-      </c>
-      <c r="K5" s="10">
-        <f>$J$26+$J$25*B5</f>
-        <v>93.565563094818472</v>
-      </c>
-      <c r="L5" s="12">
-        <f t="shared" si="0"/>
         <v>0.17443690518152266</v>
       </c>
       <c r="M5" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>3.0428233889307526E-2</v>
       </c>
     </row>
@@ -8135,43 +8131,43 @@
         <v>96.73</v>
       </c>
       <c r="D6" s="4">
+        <f t="shared" si="2"/>
+        <v>141.22579999999999</v>
+      </c>
+      <c r="E6" s="4">
+        <f t="shared" si="3"/>
+        <v>2.1315999999999997</v>
+      </c>
+      <c r="F6" s="4">
+        <f t="shared" si="4"/>
+        <v>9356.6929</v>
+      </c>
+      <c r="G6" s="7">
+        <f t="shared" si="5"/>
+        <v>0.26399999999999979</v>
+      </c>
+      <c r="H6" s="7">
+        <f t="shared" si="6"/>
+        <v>4.569500000000005</v>
+      </c>
+      <c r="I6" s="8">
+        <f t="shared" si="7"/>
+        <v>6.9695999999999883E-2</v>
+      </c>
+      <c r="J6" s="9">
+        <f t="shared" si="8"/>
+        <v>1.2063480000000004</v>
+      </c>
+      <c r="K6" s="10">
+        <f t="shared" si="0"/>
+        <v>96.10663464927741</v>
+      </c>
+      <c r="L6" s="12">
         <f t="shared" si="1"/>
-        <v>141.22579999999999</v>
-      </c>
-      <c r="E6" s="4">
-        <f t="shared" si="2"/>
-        <v>2.1315999999999997</v>
-      </c>
-      <c r="F6" s="4">
-        <f t="shared" si="3"/>
-        <v>9356.6929</v>
-      </c>
-      <c r="G6" s="7">
-        <f>B6-B$23</f>
-        <v>0.26399999999999979</v>
-      </c>
-      <c r="H6" s="7">
-        <f t="shared" si="4"/>
-        <v>4.569500000000005</v>
-      </c>
-      <c r="I6" s="8">
-        <f t="shared" si="5"/>
-        <v>6.9695999999999883E-2</v>
-      </c>
-      <c r="J6" s="9">
-        <f t="shared" si="6"/>
-        <v>1.2063480000000004</v>
-      </c>
-      <c r="K6" s="10">
-        <f>$J$26+$J$25*B6</f>
-        <v>96.10663464927741</v>
-      </c>
-      <c r="L6" s="12">
-        <f t="shared" si="0"/>
         <v>0.6233653507225938</v>
       </c>
       <c r="M6" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.38858436048150236</v>
       </c>
     </row>
@@ -8186,43 +8182,43 @@
         <v>94.45</v>
       </c>
       <c r="D7" s="4">
+        <f t="shared" si="2"/>
+        <v>128.45200000000003</v>
+      </c>
+      <c r="E7" s="4">
+        <f t="shared" si="3"/>
+        <v>1.8496000000000004</v>
+      </c>
+      <c r="F7" s="4">
+        <f t="shared" si="4"/>
+        <v>8920.8024999999998</v>
+      </c>
+      <c r="G7" s="7">
+        <f t="shared" si="5"/>
+        <v>0.16399999999999992</v>
+      </c>
+      <c r="H7" s="7">
+        <f t="shared" si="6"/>
+        <v>2.2895000000000039</v>
+      </c>
+      <c r="I7" s="8">
+        <f t="shared" si="7"/>
+        <v>2.6895999999999975E-2</v>
+      </c>
+      <c r="J7" s="9">
+        <f t="shared" si="8"/>
+        <v>0.37547800000000048</v>
+      </c>
+      <c r="K7" s="10">
+        <f t="shared" si="0"/>
+        <v>94.611886676066277</v>
+      </c>
+      <c r="L7" s="12">
         <f t="shared" si="1"/>
-        <v>128.45200000000003</v>
-      </c>
-      <c r="E7" s="4">
-        <f t="shared" si="2"/>
-        <v>1.8496000000000004</v>
-      </c>
-      <c r="F7" s="4">
-        <f t="shared" si="3"/>
-        <v>8920.8024999999998</v>
-      </c>
-      <c r="G7" s="7">
-        <f>B7-B$23</f>
-        <v>0.16399999999999992</v>
-      </c>
-      <c r="H7" s="7">
-        <f t="shared" si="4"/>
-        <v>2.2895000000000039</v>
-      </c>
-      <c r="I7" s="8">
-        <f t="shared" si="5"/>
-        <v>2.6895999999999975E-2</v>
-      </c>
-      <c r="J7" s="9">
-        <f t="shared" si="6"/>
-        <v>0.37547800000000048</v>
-      </c>
-      <c r="K7" s="10">
-        <f>$J$26+$J$25*B7</f>
-        <v>94.611886676066277</v>
-      </c>
-      <c r="L7" s="12">
-        <f t="shared" si="0"/>
         <v>-0.16188667606627405</v>
       </c>
       <c r="M7" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.6207295887786745E-2</v>
       </c>
     </row>
@@ -8237,43 +8233,43 @@
         <v>87.59</v>
       </c>
       <c r="D8" s="4">
+        <f t="shared" si="2"/>
+        <v>76.203299999999999</v>
+      </c>
+      <c r="E8" s="4">
+        <f t="shared" si="3"/>
+        <v>0.75690000000000002</v>
+      </c>
+      <c r="F8" s="4">
+        <f t="shared" si="4"/>
+        <v>7672.0081000000009</v>
+      </c>
+      <c r="G8" s="7">
+        <f t="shared" si="5"/>
+        <v>-0.32600000000000018</v>
+      </c>
+      <c r="H8" s="7">
+        <f t="shared" si="6"/>
+        <v>-4.5704999999999956</v>
+      </c>
+      <c r="I8" s="8">
+        <f t="shared" si="7"/>
+        <v>0.10627600000000012</v>
+      </c>
+      <c r="J8" s="9">
+        <f t="shared" si="8"/>
+        <v>1.4899829999999994</v>
+      </c>
+      <c r="K8" s="10">
+        <f t="shared" si="0"/>
+        <v>87.287621607331687</v>
+      </c>
+      <c r="L8" s="12">
         <f t="shared" si="1"/>
-        <v>76.203299999999999</v>
-      </c>
-      <c r="E8" s="4">
-        <f t="shared" si="2"/>
-        <v>0.75690000000000002</v>
-      </c>
-      <c r="F8" s="4">
-        <f t="shared" si="3"/>
-        <v>7672.0081000000009</v>
-      </c>
-      <c r="G8" s="7">
-        <f>B8-B$23</f>
-        <v>-0.32600000000000018</v>
-      </c>
-      <c r="H8" s="7">
-        <f t="shared" si="4"/>
-        <v>-4.5704999999999956</v>
-      </c>
-      <c r="I8" s="8">
-        <f t="shared" si="5"/>
-        <v>0.10627600000000012</v>
-      </c>
-      <c r="J8" s="9">
-        <f t="shared" si="6"/>
-        <v>1.4899829999999994</v>
-      </c>
-      <c r="K8" s="10">
-        <f>$J$26+$J$25*B8</f>
-        <v>87.287621607331687</v>
-      </c>
-      <c r="L8" s="12">
-        <f t="shared" si="0"/>
         <v>0.30237839266831656</v>
       </c>
       <c r="M8" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>9.1432692352674635E-2</v>
       </c>
     </row>
@@ -8288,43 +8284,43 @@
         <v>91.77</v>
       </c>
       <c r="D9" s="4">
+        <f t="shared" si="2"/>
+        <v>112.8771</v>
+      </c>
+      <c r="E9" s="4">
+        <f t="shared" si="3"/>
+        <v>1.5128999999999999</v>
+      </c>
+      <c r="F9" s="4">
+        <f t="shared" si="4"/>
+        <v>8421.7328999999991</v>
+      </c>
+      <c r="G9" s="7">
+        <f t="shared" si="5"/>
+        <v>3.3999999999999808E-2</v>
+      </c>
+      <c r="H9" s="7">
+        <f t="shared" si="6"/>
+        <v>-0.39050000000000296</v>
+      </c>
+      <c r="I9" s="8">
+        <f t="shared" si="7"/>
+        <v>1.1559999999999869E-3</v>
+      </c>
+      <c r="J9" s="9">
+        <f t="shared" si="8"/>
+        <v>-1.3277000000000025E-2</v>
+      </c>
+      <c r="K9" s="10">
+        <f t="shared" si="0"/>
+        <v>92.668714310891787</v>
+      </c>
+      <c r="L9" s="12">
         <f t="shared" si="1"/>
-        <v>112.8771</v>
-      </c>
-      <c r="E9" s="4">
-        <f t="shared" si="2"/>
-        <v>1.5128999999999999</v>
-      </c>
-      <c r="F9" s="4">
-        <f t="shared" si="3"/>
-        <v>8421.7328999999991</v>
-      </c>
-      <c r="G9" s="7">
-        <f>B9-B$23</f>
-        <v>3.3999999999999808E-2</v>
-      </c>
-      <c r="H9" s="7">
-        <f t="shared" si="4"/>
-        <v>-0.39050000000000296</v>
-      </c>
-      <c r="I9" s="8">
-        <f t="shared" si="5"/>
-        <v>1.1559999999999869E-3</v>
-      </c>
-      <c r="J9" s="9">
-        <f t="shared" si="6"/>
-        <v>-1.3277000000000025E-2</v>
-      </c>
-      <c r="K9" s="10">
-        <f>$J$26+$J$25*B9</f>
-        <v>92.668714310891787</v>
-      </c>
-      <c r="L9" s="12">
-        <f t="shared" si="0"/>
         <v>-0.89871431089179055</v>
       </c>
       <c r="M9" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.80768741260170596</v>
       </c>
     </row>
@@ -8339,43 +8335,43 @@
         <v>99.42</v>
       </c>
       <c r="D10" s="4">
+        <f t="shared" si="2"/>
+        <v>154.101</v>
+      </c>
+      <c r="E10" s="4">
+        <f t="shared" si="3"/>
+        <v>2.4025000000000003</v>
+      </c>
+      <c r="F10" s="4">
+        <f t="shared" si="4"/>
+        <v>9884.3364000000001</v>
+      </c>
+      <c r="G10" s="7">
+        <f t="shared" si="5"/>
+        <v>0.35399999999999987</v>
+      </c>
+      <c r="H10" s="7">
+        <f t="shared" si="6"/>
+        <v>7.2595000000000027</v>
+      </c>
+      <c r="I10" s="8">
+        <f t="shared" si="7"/>
+        <v>0.1253159999999999</v>
+      </c>
+      <c r="J10" s="9">
+        <f t="shared" si="8"/>
+        <v>2.5698630000000002</v>
+      </c>
+      <c r="K10" s="10">
+        <f t="shared" si="0"/>
+        <v>97.451907825167439</v>
+      </c>
+      <c r="L10" s="12">
         <f t="shared" si="1"/>
-        <v>154.101</v>
-      </c>
-      <c r="E10" s="4">
-        <f t="shared" si="2"/>
-        <v>2.4025000000000003</v>
-      </c>
-      <c r="F10" s="4">
-        <f t="shared" si="3"/>
-        <v>9884.3364000000001</v>
-      </c>
-      <c r="G10" s="7">
-        <f>B10-B$23</f>
-        <v>0.35399999999999987</v>
-      </c>
-      <c r="H10" s="7">
-        <f t="shared" si="4"/>
-        <v>7.2595000000000027</v>
-      </c>
-      <c r="I10" s="8">
-        <f t="shared" si="5"/>
-        <v>0.1253159999999999</v>
-      </c>
-      <c r="J10" s="9">
-        <f t="shared" si="6"/>
-        <v>2.5698630000000002</v>
-      </c>
-      <c r="K10" s="10">
-        <f>$J$26+$J$25*B10</f>
-        <v>97.451907825167439</v>
-      </c>
-      <c r="L10" s="12">
-        <f t="shared" si="0"/>
         <v>1.968092174832563</v>
       </c>
       <c r="M10" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>3.8733868086371679</v>
       </c>
     </row>
@@ -8390,43 +8386,43 @@
         <v>93.65</v>
       </c>
       <c r="D11" s="4">
+        <f t="shared" si="2"/>
+        <v>131.11000000000001</v>
+      </c>
+      <c r="E11" s="4">
+        <f t="shared" si="3"/>
+        <v>1.9599999999999997</v>
+      </c>
+      <c r="F11" s="4">
+        <f t="shared" si="4"/>
+        <v>8770.3225000000002</v>
+      </c>
+      <c r="G11" s="7">
+        <f t="shared" si="5"/>
+        <v>0.20399999999999974</v>
+      </c>
+      <c r="H11" s="7">
+        <f t="shared" si="6"/>
+        <v>1.4895000000000067</v>
+      </c>
+      <c r="I11" s="8">
+        <f t="shared" si="7"/>
+        <v>4.1615999999999896E-2</v>
+      </c>
+      <c r="J11" s="9">
+        <f t="shared" si="8"/>
+        <v>0.30385800000000096</v>
+      </c>
+      <c r="K11" s="10">
+        <f t="shared" si="0"/>
+        <v>95.209785865350725</v>
+      </c>
+      <c r="L11" s="12">
         <f t="shared" si="1"/>
-        <v>131.11000000000001</v>
-      </c>
-      <c r="E11" s="4">
-        <f t="shared" si="2"/>
-        <v>1.9599999999999997</v>
-      </c>
-      <c r="F11" s="4">
-        <f t="shared" si="3"/>
-        <v>8770.3225000000002</v>
-      </c>
-      <c r="G11" s="7">
-        <f>B11-B$23</f>
-        <v>0.20399999999999974</v>
-      </c>
-      <c r="H11" s="7">
-        <f t="shared" si="4"/>
-        <v>1.4895000000000067</v>
-      </c>
-      <c r="I11" s="8">
-        <f t="shared" si="5"/>
-        <v>4.1615999999999896E-2</v>
-      </c>
-      <c r="J11" s="9">
-        <f t="shared" si="6"/>
-        <v>0.30385800000000096</v>
-      </c>
-      <c r="K11" s="10">
-        <f>$J$26+$J$25*B11</f>
-        <v>95.209785865350725</v>
-      </c>
-      <c r="L11" s="12">
-        <f t="shared" si="0"/>
         <v>-1.5597858653507188</v>
       </c>
       <c r="M11" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.4329319457478906</v>
       </c>
     </row>
@@ -8441,43 +8437,43 @@
         <v>93.54</v>
       </c>
       <c r="D12" s="4">
+        <f t="shared" si="2"/>
+        <v>111.3126</v>
+      </c>
+      <c r="E12" s="4">
+        <f t="shared" si="3"/>
+        <v>1.4160999999999999</v>
+      </c>
+      <c r="F12" s="4">
+        <f t="shared" si="4"/>
+        <v>8749.731600000001</v>
+      </c>
+      <c r="G12" s="7">
+        <f t="shared" si="5"/>
+        <v>-6.0000000000002274E-3</v>
+      </c>
+      <c r="H12" s="7">
+        <f t="shared" si="6"/>
+        <v>1.3795000000000073</v>
+      </c>
+      <c r="I12" s="8">
+        <f t="shared" si="7"/>
+        <v>3.6000000000002732E-5</v>
+      </c>
+      <c r="J12" s="9">
+        <f t="shared" si="8"/>
+        <v>-8.277000000000357E-3</v>
+      </c>
+      <c r="K12" s="10">
+        <f t="shared" si="0"/>
+        <v>92.070815121607339</v>
+      </c>
+      <c r="L12" s="12">
         <f t="shared" si="1"/>
-        <v>111.3126</v>
-      </c>
-      <c r="E12" s="4">
-        <f t="shared" si="2"/>
-        <v>1.4160999999999999</v>
-      </c>
-      <c r="F12" s="4">
-        <f t="shared" si="3"/>
-        <v>8749.731600000001</v>
-      </c>
-      <c r="G12" s="7">
-        <f>B12-B$23</f>
-        <v>-6.0000000000002274E-3</v>
-      </c>
-      <c r="H12" s="7">
-        <f t="shared" si="4"/>
-        <v>1.3795000000000073</v>
-      </c>
-      <c r="I12" s="8">
-        <f t="shared" si="5"/>
-        <v>3.6000000000002732E-5</v>
-      </c>
-      <c r="J12" s="9">
-        <f t="shared" si="6"/>
-        <v>-8.277000000000357E-3</v>
-      </c>
-      <c r="K12" s="10">
-        <f>$J$26+$J$25*B12</f>
-        <v>92.070815121607339</v>
-      </c>
-      <c r="L12" s="12">
-        <f t="shared" si="0"/>
         <v>1.4691848783926673</v>
       </c>
       <c r="M12" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.1585042068976765</v>
       </c>
     </row>
@@ -8492,43 +8488,43 @@
         <v>92.52</v>
       </c>
       <c r="D13" s="4">
+        <f t="shared" si="2"/>
+        <v>106.39799999999998</v>
+      </c>
+      <c r="E13" s="4">
+        <f t="shared" si="3"/>
+        <v>1.3224999999999998</v>
+      </c>
+      <c r="F13" s="4">
+        <f t="shared" si="4"/>
+        <v>8559.9503999999997</v>
+      </c>
+      <c r="G13" s="7">
+        <f t="shared" si="5"/>
+        <v>-4.6000000000000263E-2</v>
+      </c>
+      <c r="H13" s="7">
+        <f t="shared" si="6"/>
+        <v>0.35949999999999704</v>
+      </c>
+      <c r="I13" s="8">
+        <f t="shared" si="7"/>
+        <v>2.1160000000000241E-3</v>
+      </c>
+      <c r="J13" s="9">
+        <f t="shared" si="8"/>
+        <v>-1.6536999999999958E-2</v>
+      </c>
+      <c r="K13" s="10">
+        <f t="shared" si="0"/>
+        <v>91.472915932322877</v>
+      </c>
+      <c r="L13" s="12">
         <f t="shared" si="1"/>
-        <v>106.39799999999998</v>
-      </c>
-      <c r="E13" s="4">
-        <f t="shared" si="2"/>
-        <v>1.3224999999999998</v>
-      </c>
-      <c r="F13" s="4">
-        <f t="shared" si="3"/>
-        <v>8559.9503999999997</v>
-      </c>
-      <c r="G13" s="7">
-        <f>B13-B$23</f>
-        <v>-4.6000000000000263E-2</v>
-      </c>
-      <c r="H13" s="7">
-        <f t="shared" si="4"/>
-        <v>0.35949999999999704</v>
-      </c>
-      <c r="I13" s="8">
-        <f t="shared" si="5"/>
-        <v>2.1160000000000241E-3</v>
-      </c>
-      <c r="J13" s="9">
-        <f t="shared" si="6"/>
-        <v>-1.6536999999999958E-2</v>
-      </c>
-      <c r="K13" s="10">
-        <f>$J$26+$J$25*B13</f>
-        <v>91.472915932322877</v>
-      </c>
-      <c r="L13" s="12">
-        <f t="shared" si="0"/>
         <v>1.0470840676771189</v>
       </c>
       <c r="M13" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.0963850447832613</v>
       </c>
     </row>
@@ -8543,43 +8539,43 @@
         <v>90.56</v>
       </c>
       <c r="D14" s="4">
+        <f t="shared" si="2"/>
+        <v>88.748800000000003</v>
+      </c>
+      <c r="E14" s="4">
+        <f t="shared" si="3"/>
+        <v>0.96039999999999992</v>
+      </c>
+      <c r="F14" s="4">
+        <f t="shared" si="4"/>
+        <v>8201.1136000000006</v>
+      </c>
+      <c r="G14" s="7">
+        <f t="shared" si="5"/>
+        <v>-0.21600000000000019</v>
+      </c>
+      <c r="H14" s="7">
+        <f t="shared" si="6"/>
+        <v>-1.6004999999999967</v>
+      </c>
+      <c r="I14" s="8">
+        <f t="shared" si="7"/>
+        <v>4.6656000000000086E-2</v>
+      </c>
+      <c r="J14" s="9">
+        <f t="shared" si="8"/>
+        <v>0.34570799999999957</v>
+      </c>
+      <c r="K14" s="10">
+        <f t="shared" si="0"/>
+        <v>88.931844377863939</v>
+      </c>
+      <c r="L14" s="12">
         <f t="shared" si="1"/>
-        <v>88.748800000000003</v>
-      </c>
-      <c r="E14" s="4">
-        <f t="shared" si="2"/>
-        <v>0.96039999999999992</v>
-      </c>
-      <c r="F14" s="4">
-        <f t="shared" si="3"/>
-        <v>8201.1136000000006</v>
-      </c>
-      <c r="G14" s="7">
-        <f>B14-B$23</f>
-        <v>-0.21600000000000019</v>
-      </c>
-      <c r="H14" s="7">
-        <f t="shared" si="4"/>
-        <v>-1.6004999999999967</v>
-      </c>
-      <c r="I14" s="8">
-        <f t="shared" si="5"/>
-        <v>4.6656000000000086E-2</v>
-      </c>
-      <c r="J14" s="9">
-        <f t="shared" si="6"/>
-        <v>0.34570799999999957</v>
-      </c>
-      <c r="K14" s="10">
-        <f>$J$26+$J$25*B14</f>
-        <v>88.931844377863939</v>
-      </c>
-      <c r="L14" s="12">
-        <f t="shared" si="0"/>
         <v>1.6281556221360631</v>
       </c>
       <c r="M14" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.6508907298932707</v>
       </c>
     </row>
@@ -8594,43 +8590,43 @@
         <v>89.54</v>
       </c>
       <c r="D15" s="4">
+        <f t="shared" si="2"/>
+        <v>90.435400000000001</v>
+      </c>
+      <c r="E15" s="4">
+        <f t="shared" si="3"/>
+        <v>1.0201</v>
+      </c>
+      <c r="F15" s="4">
+        <f t="shared" si="4"/>
+        <v>8017.4116000000013</v>
+      </c>
+      <c r="G15" s="7">
+        <f t="shared" si="5"/>
+        <v>-0.18600000000000017</v>
+      </c>
+      <c r="H15" s="7">
+        <f t="shared" si="6"/>
+        <v>-2.6204999999999927</v>
+      </c>
+      <c r="I15" s="8">
+        <f t="shared" si="7"/>
+        <v>3.4596000000000064E-2</v>
+      </c>
+      <c r="J15" s="9">
+        <f t="shared" si="8"/>
+        <v>0.4874129999999991</v>
+      </c>
+      <c r="K15" s="10">
+        <f t="shared" si="0"/>
+        <v>89.380268769827282</v>
+      </c>
+      <c r="L15" s="12">
         <f t="shared" si="1"/>
-        <v>90.435400000000001</v>
-      </c>
-      <c r="E15" s="4">
-        <f t="shared" si="2"/>
-        <v>1.0201</v>
-      </c>
-      <c r="F15" s="4">
-        <f t="shared" si="3"/>
-        <v>8017.4116000000013</v>
-      </c>
-      <c r="G15" s="7">
-        <f>B15-B$23</f>
-        <v>-0.18600000000000017</v>
-      </c>
-      <c r="H15" s="7">
-        <f t="shared" si="4"/>
-        <v>-2.6204999999999927</v>
-      </c>
-      <c r="I15" s="8">
-        <f t="shared" si="5"/>
-        <v>3.4596000000000064E-2</v>
-      </c>
-      <c r="J15" s="9">
-        <f t="shared" si="6"/>
-        <v>0.4874129999999991</v>
-      </c>
-      <c r="K15" s="10">
-        <f>$J$26+$J$25*B15</f>
-        <v>89.380268769827282</v>
-      </c>
-      <c r="L15" s="12">
-        <f t="shared" si="0"/>
         <v>0.15973123017272428</v>
       </c>
       <c r="M15" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.5514065892491822E-2</v>
       </c>
     </row>
@@ -8645,43 +8641,43 @@
         <v>89.85</v>
       </c>
       <c r="D16" s="4">
+        <f t="shared" si="2"/>
+        <v>99.733500000000006</v>
+      </c>
+      <c r="E16" s="4">
+        <f t="shared" si="3"/>
+        <v>1.2321000000000002</v>
+      </c>
+      <c r="F16" s="4">
+        <f t="shared" si="4"/>
+        <v>8073.0224999999991</v>
+      </c>
+      <c r="G16" s="7">
+        <f t="shared" si="5"/>
+        <v>-8.6000000000000076E-2</v>
+      </c>
+      <c r="H16" s="7">
+        <f t="shared" si="6"/>
+        <v>-2.3105000000000047</v>
+      </c>
+      <c r="I16" s="8">
+        <f t="shared" si="7"/>
+        <v>7.3960000000000128E-3</v>
+      </c>
+      <c r="J16" s="9">
+        <f t="shared" si="8"/>
+        <v>0.19870300000000057</v>
+      </c>
+      <c r="K16" s="10">
+        <f t="shared" si="0"/>
+        <v>90.875016743038429</v>
+      </c>
+      <c r="L16" s="12">
         <f t="shared" si="1"/>
-        <v>99.733500000000006</v>
-      </c>
-      <c r="E16" s="4">
-        <f t="shared" si="2"/>
-        <v>1.2321000000000002</v>
-      </c>
-      <c r="F16" s="4">
-        <f t="shared" si="3"/>
-        <v>8073.0224999999991</v>
-      </c>
-      <c r="G16" s="7">
-        <f>B16-B$23</f>
-        <v>-8.6000000000000076E-2</v>
-      </c>
-      <c r="H16" s="7">
-        <f t="shared" si="4"/>
-        <v>-2.3105000000000047</v>
-      </c>
-      <c r="I16" s="8">
-        <f t="shared" si="5"/>
-        <v>7.3960000000000128E-3</v>
-      </c>
-      <c r="J16" s="9">
-        <f t="shared" si="6"/>
-        <v>0.19870300000000057</v>
-      </c>
-      <c r="K16" s="10">
-        <f>$J$26+$J$25*B16</f>
-        <v>90.875016743038429</v>
-      </c>
-      <c r="L16" s="12">
-        <f t="shared" si="0"/>
         <v>-1.0250167430384352</v>
       </c>
       <c r="M16" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.0506593235091215</v>
       </c>
     </row>
@@ -8696,43 +8692,43 @@
         <v>90.39</v>
       </c>
       <c r="D17" s="4">
+        <f t="shared" si="2"/>
+        <v>108.468</v>
+      </c>
+      <c r="E17" s="4">
+        <f t="shared" si="3"/>
+        <v>1.44</v>
+      </c>
+      <c r="F17" s="4">
+        <f t="shared" si="4"/>
+        <v>8170.3521000000001</v>
+      </c>
+      <c r="G17" s="7">
+        <f t="shared" si="5"/>
+        <v>3.9999999999997815E-3</v>
+      </c>
+      <c r="H17" s="7">
+        <f t="shared" si="6"/>
+        <v>-1.7704999999999984</v>
+      </c>
+      <c r="I17" s="8">
+        <f t="shared" si="7"/>
+        <v>1.5999999999998251E-5</v>
+      </c>
+      <c r="J17" s="9">
+        <f t="shared" si="8"/>
+        <v>-7.0819999999996068E-3</v>
+      </c>
+      <c r="K17" s="10">
+        <f t="shared" si="0"/>
+        <v>92.220289918928444</v>
+      </c>
+      <c r="L17" s="12">
         <f t="shared" si="1"/>
-        <v>108.468</v>
-      </c>
-      <c r="E17" s="4">
-        <f t="shared" si="2"/>
-        <v>1.44</v>
-      </c>
-      <c r="F17" s="4">
-        <f t="shared" si="3"/>
-        <v>8170.3521000000001</v>
-      </c>
-      <c r="G17" s="7">
-        <f>B17-B$23</f>
-        <v>3.9999999999997815E-3</v>
-      </c>
-      <c r="H17" s="7">
-        <f t="shared" si="4"/>
-        <v>-1.7704999999999984</v>
-      </c>
-      <c r="I17" s="8">
-        <f t="shared" si="5"/>
-        <v>1.5999999999998251E-5</v>
-      </c>
-      <c r="J17" s="9">
-        <f t="shared" si="6"/>
-        <v>-7.0819999999996068E-3</v>
-      </c>
-      <c r="K17" s="10">
-        <f>$J$26+$J$25*B17</f>
-        <v>92.220289918928444</v>
-      </c>
-      <c r="L17" s="12">
-        <f t="shared" si="0"/>
         <v>-1.8302899189284432</v>
       </c>
       <c r="M17" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>3.3499611873310871</v>
       </c>
     </row>
@@ -8747,43 +8743,43 @@
         <v>93.25</v>
       </c>
       <c r="D18" s="4">
+        <f t="shared" si="2"/>
+        <v>117.495</v>
+      </c>
+      <c r="E18" s="4">
+        <f t="shared" si="3"/>
+        <v>1.5876000000000001</v>
+      </c>
+      <c r="F18" s="4">
+        <f t="shared" si="4"/>
+        <v>8695.5625</v>
+      </c>
+      <c r="G18" s="7">
+        <f t="shared" si="5"/>
+        <v>6.3999999999999835E-2</v>
+      </c>
+      <c r="H18" s="7">
+        <f t="shared" si="6"/>
+        <v>1.089500000000001</v>
+      </c>
+      <c r="I18" s="8">
+        <f t="shared" si="7"/>
+        <v>4.095999999999979E-3</v>
+      </c>
+      <c r="J18" s="9">
+        <f t="shared" si="8"/>
+        <v>6.9727999999999887E-2</v>
+      </c>
+      <c r="K18" s="10">
+        <f t="shared" si="0"/>
+        <v>93.117138702855129</v>
+      </c>
+      <c r="L18" s="12">
         <f t="shared" si="1"/>
-        <v>117.495</v>
-      </c>
-      <c r="E18" s="4">
-        <f t="shared" si="2"/>
-        <v>1.5876000000000001</v>
-      </c>
-      <c r="F18" s="4">
-        <f t="shared" si="3"/>
-        <v>8695.5625</v>
-      </c>
-      <c r="G18" s="7">
-        <f>B18-B$23</f>
-        <v>6.3999999999999835E-2</v>
-      </c>
-      <c r="H18" s="7">
-        <f t="shared" si="4"/>
-        <v>1.089500000000001</v>
-      </c>
-      <c r="I18" s="8">
-        <f t="shared" si="5"/>
-        <v>4.095999999999979E-3</v>
-      </c>
-      <c r="J18" s="9">
-        <f t="shared" si="6"/>
-        <v>6.9727999999999887E-2</v>
-      </c>
-      <c r="K18" s="10">
-        <f>$J$26+$J$25*B18</f>
-        <v>93.117138702855129</v>
-      </c>
-      <c r="L18" s="12">
-        <f t="shared" si="0"/>
         <v>0.1328612971448706</v>
       </c>
       <c r="M18" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.7652124279017602E-2</v>
       </c>
     </row>
@@ -8798,43 +8794,43 @@
         <v>93.41</v>
       </c>
       <c r="D19" s="4">
+        <f t="shared" si="2"/>
+        <v>123.30119999999999</v>
+      </c>
+      <c r="E19" s="4">
+        <f t="shared" si="3"/>
+        <v>1.7424000000000002</v>
+      </c>
+      <c r="F19" s="4">
+        <f t="shared" si="4"/>
+        <v>8725.4280999999992</v>
+      </c>
+      <c r="G19" s="7">
+        <f t="shared" si="5"/>
+        <v>0.12399999999999989</v>
+      </c>
+      <c r="H19" s="7">
+        <f t="shared" si="6"/>
+        <v>1.2494999999999976</v>
+      </c>
+      <c r="I19" s="8">
+        <f t="shared" si="7"/>
+        <v>1.5375999999999973E-2</v>
+      </c>
+      <c r="J19" s="9">
+        <f t="shared" si="8"/>
+        <v>0.15493799999999958</v>
+      </c>
+      <c r="K19" s="10">
+        <f t="shared" si="0"/>
+        <v>94.013987486781815</v>
+      </c>
+      <c r="L19" s="12">
         <f t="shared" si="1"/>
-        <v>123.30119999999999</v>
-      </c>
-      <c r="E19" s="4">
-        <f t="shared" si="2"/>
-        <v>1.7424000000000002</v>
-      </c>
-      <c r="F19" s="4">
-        <f t="shared" si="3"/>
-        <v>8725.4280999999992</v>
-      </c>
-      <c r="G19" s="7">
-        <f>B19-B$23</f>
-        <v>0.12399999999999989</v>
-      </c>
-      <c r="H19" s="7">
-        <f t="shared" si="4"/>
-        <v>1.2494999999999976</v>
-      </c>
-      <c r="I19" s="8">
-        <f t="shared" si="5"/>
-        <v>1.5375999999999973E-2</v>
-      </c>
-      <c r="J19" s="9">
-        <f t="shared" si="6"/>
-        <v>0.15493799999999958</v>
-      </c>
-      <c r="K19" s="10">
-        <f>$J$26+$J$25*B19</f>
-        <v>94.013987486781815</v>
-      </c>
-      <c r="L19" s="12">
-        <f t="shared" si="0"/>
         <v>-0.60398748678181846</v>
       </c>
       <c r="M19" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.36480088418901735</v>
       </c>
     </row>
@@ -8849,43 +8845,43 @@
         <v>94.98</v>
       </c>
       <c r="D20" s="4">
+        <f t="shared" si="2"/>
+        <v>135.82140000000001</v>
+      </c>
+      <c r="E20" s="4">
+        <f t="shared" si="3"/>
+        <v>2.0448999999999997</v>
+      </c>
+      <c r="F20" s="4">
+        <f t="shared" si="4"/>
+        <v>9021.2004000000015</v>
+      </c>
+      <c r="G20" s="7">
+        <f t="shared" si="5"/>
+        <v>0.23399999999999976</v>
+      </c>
+      <c r="H20" s="7">
+        <f t="shared" si="6"/>
+        <v>2.819500000000005</v>
+      </c>
+      <c r="I20" s="8">
+        <f t="shared" si="7"/>
+        <v>5.4755999999999888E-2</v>
+      </c>
+      <c r="J20" s="9">
+        <f t="shared" si="8"/>
+        <v>0.65976300000000054</v>
+      </c>
+      <c r="K20" s="10">
+        <f t="shared" si="0"/>
+        <v>95.658210257314067</v>
+      </c>
+      <c r="L20" s="12">
         <f t="shared" si="1"/>
-        <v>135.82140000000001</v>
-      </c>
-      <c r="E20" s="4">
-        <f t="shared" si="2"/>
-        <v>2.0448999999999997</v>
-      </c>
-      <c r="F20" s="4">
-        <f t="shared" si="3"/>
-        <v>9021.2004000000015</v>
-      </c>
-      <c r="G20" s="7">
-        <f>B20-B$23</f>
-        <v>0.23399999999999976</v>
-      </c>
-      <c r="H20" s="7">
-        <f t="shared" si="4"/>
-        <v>2.819500000000005</v>
-      </c>
-      <c r="I20" s="8">
-        <f t="shared" si="5"/>
-        <v>5.4755999999999888E-2</v>
-      </c>
-      <c r="J20" s="9">
-        <f t="shared" si="6"/>
-        <v>0.65976300000000054</v>
-      </c>
-      <c r="K20" s="10">
-        <f>$J$26+$J$25*B20</f>
-        <v>95.658210257314067</v>
-      </c>
-      <c r="L20" s="12">
-        <f t="shared" si="0"/>
         <v>-0.67821025731406337</v>
       </c>
       <c r="M20" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.45996915312600806</v>
       </c>
     </row>
@@ -8900,11 +8896,11 @@
         <v>87.33</v>
       </c>
       <c r="D21" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>82.963499999999996</v>
       </c>
       <c r="E21" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.90249999999999997</v>
       </c>
       <c r="F21" s="4">
@@ -8912,31 +8908,31 @@
         <v>7626.5288999999993</v>
       </c>
       <c r="G21" s="7">
-        <f>B21-B$23</f>
+        <f t="shared" si="5"/>
         <v>-0.24600000000000022</v>
       </c>
       <c r="H21" s="7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>-4.8305000000000007</v>
       </c>
       <c r="I21" s="8">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>6.0516000000000104E-2</v>
       </c>
       <c r="J21" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1.1883030000000012</v>
       </c>
       <c r="K21" s="10">
-        <f>$J$26+$J$25*B21</f>
+        <f t="shared" si="0"/>
         <v>88.483419985900596</v>
       </c>
       <c r="L21" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-1.153419985900598</v>
       </c>
       <c r="M21" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.3303776638749358</v>
       </c>
     </row>
@@ -8973,9 +8969,9 @@
         <f>AVERAGE(C2:C21)</f>
         <v>92.160499999999999</v>
       </c>
-      <c r="D23" s="33"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
       <c r="G23" s="1"/>
       <c r="I23" s="9">
         <f>SUM(I2:I21)</f>
@@ -9306,10 +9302,10 @@
         <f t="shared" si="2"/>
         <v>14400</v>
       </c>
-      <c r="I4" s="37" t="s">
+      <c r="I4" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="J4" s="37"/>
+      <c r="J4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
@@ -9336,10 +9332,10 @@
         <f t="shared" si="2"/>
         <v>302500</v>
       </c>
-      <c r="I5" s="34" t="s">
+      <c r="I5" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="34">
+      <c r="J5">
         <v>0.99562903793909374</v>
       </c>
     </row>
@@ -9368,10 +9364,10 @@
         <f t="shared" si="2"/>
         <v>87025</v>
       </c>
-      <c r="I6" s="34" t="s">
+      <c r="I6" t="s">
         <v>47</v>
       </c>
-      <c r="J6" s="34">
+      <c r="J6">
         <v>0.99127718118752528</v>
       </c>
     </row>
@@ -9400,10 +9396,10 @@
         <f t="shared" si="2"/>
         <v>40000</v>
       </c>
-      <c r="I7" s="34" t="s">
+      <c r="I7" t="s">
         <v>48</v>
       </c>
-      <c r="J7" s="34">
+      <c r="J7">
         <v>0.9889817025526636</v>
       </c>
     </row>
@@ -9432,10 +9428,10 @@
         <f t="shared" si="2"/>
         <v>140625</v>
       </c>
-      <c r="I8" s="34" t="s">
+      <c r="I8" t="s">
         <v>49</v>
       </c>
-      <c r="J8" s="34">
+      <c r="J8">
         <v>1.6742798818405129</v>
       </c>
     </row>
@@ -9464,10 +9460,10 @@
         <f t="shared" si="2"/>
         <v>2704</v>
       </c>
-      <c r="I9" s="35" t="s">
+      <c r="I9" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="J9" s="35">
+      <c r="J9" s="33">
         <v>25</v>
       </c>
     </row>
@@ -9551,20 +9547,20 @@
         <f t="shared" si="2"/>
         <v>169744</v>
       </c>
-      <c r="I12" s="36"/>
-      <c r="J12" s="36" t="s">
+      <c r="I12" s="34"/>
+      <c r="J12" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="K12" s="36" t="s">
+      <c r="K12" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="L12" s="36" t="s">
+      <c r="L12" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="M12" s="36" t="s">
+      <c r="M12" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="N12" s="36" t="s">
+      <c r="N12" s="34" t="s">
         <v>60</v>
       </c>
     </row>
@@ -9593,22 +9589,22 @@
         <f t="shared" si="2"/>
         <v>160000</v>
       </c>
-      <c r="I13" s="34" t="s">
+      <c r="I13" t="s">
         <v>52</v>
       </c>
-      <c r="J13" s="34">
+      <c r="J13">
         <v>5</v>
       </c>
-      <c r="K13" s="34">
+      <c r="K13">
         <v>6052.6836546680197</v>
       </c>
-      <c r="L13" s="34">
+      <c r="L13">
         <v>1210.5367309336038</v>
       </c>
-      <c r="M13" s="34">
+      <c r="M13">
         <v>431.83899258867029</v>
       </c>
-      <c r="N13" s="34">
+      <c r="N13">
         <v>7.14926629647784E-19</v>
       </c>
     </row>
@@ -9637,20 +9633,18 @@
         <f t="shared" si="2"/>
         <v>250000</v>
       </c>
-      <c r="I14" s="34" t="s">
+      <c r="I14" t="s">
         <v>53</v>
       </c>
-      <c r="J14" s="34">
+      <c r="J14">
         <v>19</v>
       </c>
-      <c r="K14" s="34">
+      <c r="K14">
         <v>53.261049331981759</v>
       </c>
-      <c r="L14" s="34">
+      <c r="L14">
         <v>2.8032131227358819</v>
       </c>
-      <c r="M14" s="34"/>
-      <c r="N14" s="34"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
@@ -9677,18 +9671,18 @@
         <f t="shared" si="2"/>
         <v>129600</v>
       </c>
-      <c r="I15" s="35" t="s">
+      <c r="I15" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="J15" s="35">
+      <c r="J15" s="33">
         <v>24</v>
       </c>
-      <c r="K15" s="35">
+      <c r="K15" s="33">
         <v>6105.9447040000014</v>
       </c>
-      <c r="L15" s="35"/>
-      <c r="M15" s="35"/>
-      <c r="N15" s="35"/>
+      <c r="L15" s="33"/>
+      <c r="M15" s="33"/>
+      <c r="N15" s="33"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6">
@@ -9741,29 +9735,29 @@
         <f t="shared" si="2"/>
         <v>160000</v>
       </c>
-      <c r="I17" s="36"/>
-      <c r="J17" s="36" t="s">
+      <c r="I17" s="34"/>
+      <c r="J17" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="K17" s="36" t="s">
+      <c r="K17" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="L17" s="36" t="s">
+      <c r="L17" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="M17" s="36" t="s">
+      <c r="M17" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="N17" s="36" t="s">
+      <c r="N17" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="O17" s="36" t="s">
+      <c r="O17" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="P17" s="36" t="s">
+      <c r="P17" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="Q17" s="36" t="s">
+      <c r="Q17" s="34" t="s">
         <v>67</v>
       </c>
     </row>
@@ -9792,31 +9786,31 @@
         <f t="shared" si="2"/>
         <v>360000</v>
       </c>
-      <c r="I18" s="34" t="s">
+      <c r="I18" t="s">
         <v>55</v>
       </c>
-      <c r="J18" s="34">
+      <c r="J18">
         <v>6.4689423071250367</v>
       </c>
-      <c r="K18" s="34">
+      <c r="K18">
         <v>1.4438373448994346</v>
       </c>
-      <c r="L18" s="34">
+      <c r="L18">
         <v>4.4803816233023177</v>
       </c>
-      <c r="M18" s="38">
+      <c r="M18" s="36">
         <v>2.5634893107229245E-4</v>
       </c>
-      <c r="N18" s="34">
+      <c r="N18">
         <v>3.446956013597493</v>
       </c>
-      <c r="O18" s="34">
+      <c r="O18">
         <v>9.4909286006525804</v>
       </c>
-      <c r="P18" s="34">
+      <c r="P18">
         <v>3.446956013597493</v>
       </c>
-      <c r="Q18" s="34">
+      <c r="Q18">
         <v>9.4909286006525804</v>
       </c>
     </row>
@@ -9845,31 +9839,31 @@
         <f t="shared" si="2"/>
         <v>342225</v>
       </c>
-      <c r="I19" s="34" t="s">
+      <c r="I19" t="s">
         <v>21</v>
       </c>
-      <c r="J19" s="34">
+      <c r="J19">
         <v>1.6561823463141032</v>
       </c>
-      <c r="K19" s="34">
+      <c r="K19">
         <v>0.26995121453257653</v>
       </c>
-      <c r="L19" s="34">
+      <c r="L19">
         <v>6.1351172254653532</v>
       </c>
-      <c r="M19" s="38">
+      <c r="M19" s="36">
         <v>6.7480108827226469E-6</v>
       </c>
-      <c r="N19" s="34">
+      <c r="N19">
         <v>1.0911679607806826</v>
       </c>
-      <c r="O19" s="34">
+      <c r="O19">
         <v>2.2211967318475239</v>
       </c>
-      <c r="P19" s="34">
+      <c r="P19">
         <v>1.0911679607806826</v>
       </c>
-      <c r="Q19" s="34">
+      <c r="Q19">
         <v>2.2211967318475239</v>
       </c>
     </row>
@@ -9898,31 +9892,31 @@
         <f t="shared" si="2"/>
         <v>291600</v>
       </c>
-      <c r="I20" s="34" t="s">
+      <c r="I20" t="s">
         <v>22</v>
       </c>
-      <c r="J20" s="34">
+      <c r="J20">
         <v>1.6656793552665167E-2</v>
       </c>
-      <c r="K20" s="34">
+      <c r="K20">
         <v>8.7005979804351159E-3</v>
       </c>
-      <c r="L20" s="34">
+      <c r="L20">
         <v>1.9144423854683332</v>
       </c>
-      <c r="M20" s="34">
+      <c r="M20">
         <v>7.0745393855091501E-2</v>
       </c>
-      <c r="N20" s="34">
+      <c r="N20">
         <v>-1.5537673081218904E-3</v>
       </c>
-      <c r="O20" s="34">
+      <c r="O20">
         <v>3.4867354413452227E-2</v>
       </c>
-      <c r="P20" s="34">
+      <c r="P20">
         <v>-1.5537673081218904E-3</v>
       </c>
-      <c r="Q20" s="34">
+      <c r="Q20">
         <v>3.4867354413452227E-2</v>
       </c>
     </row>
@@ -9951,31 +9945,31 @@
         <f t="shared" si="2"/>
         <v>62500</v>
       </c>
-      <c r="I21" s="34" t="s">
+      <c r="I21" t="s">
         <v>75</v>
       </c>
-      <c r="J21" s="34">
+      <c r="J21">
         <v>1.4819170125077801E-3</v>
       </c>
-      <c r="K21" s="34">
+      <c r="K21">
         <v>4.6289331564659396E-4</v>
       </c>
-      <c r="L21" s="34">
+      <c r="L21">
         <v>3.2014223632453187</v>
       </c>
-      <c r="M21" s="38">
+      <c r="M21" s="36">
         <v>4.6991809442873227E-3</v>
       </c>
-      <c r="N21" s="34">
+      <c r="N21">
         <v>5.1307016823464054E-4</v>
       </c>
-      <c r="O21" s="34">
+      <c r="O21">
         <v>2.4507638567809195E-3</v>
       </c>
-      <c r="P21" s="34">
+      <c r="P21">
         <v>5.1307016823464054E-4</v>
       </c>
-      <c r="Q21" s="34">
+      <c r="Q21">
         <v>2.4507638567809195E-3</v>
       </c>
     </row>
@@ -10004,31 +9998,31 @@
         <f t="shared" si="2"/>
         <v>84100</v>
       </c>
-      <c r="I22" s="34" t="s">
+      <c r="I22" t="s">
         <v>76</v>
       </c>
-      <c r="J22" s="34">
+      <c r="J22">
         <v>2.6602917254962329E-2</v>
       </c>
-      <c r="K22" s="34">
+      <c r="K22">
         <v>1.5046140782673459E-2</v>
       </c>
-      <c r="L22" s="34">
+      <c r="L22">
         <v>1.768089082723272</v>
       </c>
-      <c r="M22" s="34">
+      <c r="M22">
         <v>9.310074464953326E-2</v>
       </c>
-      <c r="N22" s="34">
+      <c r="N22">
         <v>-4.8890173291870898E-3</v>
       </c>
-      <c r="O22" s="34">
+      <c r="O22">
         <v>5.8094851839111748E-2</v>
       </c>
-      <c r="P22" s="34">
+      <c r="P22">
         <v>-4.8890173291870898E-3</v>
       </c>
-      <c r="Q22" s="34">
+      <c r="Q22">
         <v>5.8094851839111748E-2</v>
       </c>
     </row>
@@ -10057,31 +10051,31 @@
         <f t="shared" si="2"/>
         <v>260100</v>
       </c>
-      <c r="I23" s="35" t="s">
+      <c r="I23" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="J23" s="35">
+      <c r="J23" s="33">
         <v>-2.6427826384895047E-5</v>
       </c>
-      <c r="K23" s="35">
+      <c r="K23" s="33">
         <v>1.4783327801407784E-5</v>
       </c>
-      <c r="L23" s="35">
+      <c r="L23" s="33">
         <v>-1.7876777637561674</v>
       </c>
-      <c r="M23" s="35">
+      <c r="M23" s="33">
         <v>8.9790081958400783E-2</v>
       </c>
-      <c r="N23" s="35">
+      <c r="N23" s="33">
         <v>-5.7369687077444648E-5</v>
       </c>
-      <c r="O23" s="35">
+      <c r="O23" s="33">
         <v>4.5140343076545544E-6</v>
       </c>
-      <c r="P23" s="35">
+      <c r="P23" s="33">
         <v>-5.7369687077444648E-5</v>
       </c>
-      <c r="Q23" s="35">
+      <c r="Q23" s="33">
         <v>4.5140343076545544E-6</v>
       </c>
     </row>
@@ -10188,548 +10182,532 @@
     </row>
     <row r="28" spans="1:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I29" s="36" t="s">
+      <c r="I29" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="J29" s="36" t="s">
+      <c r="J29" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="K29" s="36" t="s">
+      <c r="K29" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="L29" s="36" t="s">
+      <c r="L29" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="N29" s="36" t="s">
+      <c r="N29" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="O29" s="36" t="s">
+      <c r="O29" s="34" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I30" s="34">
+      <c r="I30">
         <v>1</v>
       </c>
-      <c r="J30" s="34">
+      <c r="J30">
         <v>10.802680481694889</v>
       </c>
-      <c r="K30" s="34">
+      <c r="K30">
         <v>-0.85268048169488964</v>
       </c>
-      <c r="L30" s="34">
+      <c r="L30">
         <v>-0.57238347038382509</v>
       </c>
-      <c r="N30" s="34">
+      <c r="N30">
         <v>2</v>
       </c>
-      <c r="O30" s="34">
+      <c r="O30">
         <v>9.6</v>
       </c>
     </row>
     <row r="31" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I31" s="34">
+      <c r="I31">
         <v>2</v>
       </c>
-      <c r="J31" s="34">
+      <c r="J31">
         <v>24.23754534449824</v>
       </c>
-      <c r="K31" s="34">
+      <c r="K31">
         <v>0.21245465550175879</v>
       </c>
-      <c r="L31" s="34">
+      <c r="L31">
         <v>0.14261559356158712</v>
       </c>
-      <c r="N31" s="34">
+      <c r="N31">
         <v>6</v>
       </c>
-      <c r="O31" s="34">
+      <c r="O31">
         <v>9.9499999999999993</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I32" s="34">
+      <c r="I32">
         <v>3</v>
       </c>
-      <c r="J32" s="34">
+      <c r="J32">
         <v>31.480286087318216</v>
       </c>
-      <c r="K32" s="34">
+      <c r="K32">
         <v>0.2697139126817838</v>
       </c>
-      <c r="L32" s="34">
+      <c r="L32">
         <v>0.18105232694518308</v>
       </c>
-      <c r="N32" s="34">
+      <c r="N32">
         <v>10</v>
       </c>
-      <c r="O32" s="34">
+      <c r="O32">
         <v>10.3</v>
       </c>
     </row>
     <row r="33" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I33" s="34">
+      <c r="I33">
         <v>4</v>
       </c>
-      <c r="J33" s="34">
+      <c r="J33">
         <v>35.00842003709019</v>
       </c>
-      <c r="K33" s="34">
+      <c r="K33">
         <v>-8.4200370901896804E-3</v>
       </c>
-      <c r="L33" s="34">
+      <c r="L33">
         <v>-5.6521641504722834E-3</v>
       </c>
-      <c r="N33" s="34">
+      <c r="N33">
         <v>14</v>
       </c>
-      <c r="O33" s="34">
+      <c r="O33">
         <v>11.66</v>
       </c>
     </row>
     <row r="34" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I34" s="34">
+      <c r="I34">
         <v>5</v>
       </c>
-      <c r="J34" s="34">
+      <c r="J34">
         <v>27.532184438364546</v>
       </c>
-      <c r="K34" s="34">
+      <c r="K34">
         <v>-2.512184438364546</v>
       </c>
-      <c r="L34" s="34">
+      <c r="L34">
         <v>-1.686367728527258</v>
       </c>
-      <c r="N34" s="34">
+      <c r="N34">
         <v>18</v>
       </c>
-      <c r="O34" s="34">
+      <c r="O34">
         <v>14.38</v>
       </c>
     </row>
     <row r="35" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I35" s="34">
+      <c r="I35">
         <v>6</v>
       </c>
-      <c r="J35" s="34">
+      <c r="J35">
         <v>16.979097633604301</v>
       </c>
-      <c r="K35" s="34">
+      <c r="K35">
         <v>-0.11909763360430148</v>
       </c>
-      <c r="L35" s="34">
+      <c r="L35">
         <v>-7.9947317078760224E-2</v>
       </c>
-      <c r="N35" s="34">
+      <c r="N35">
         <v>22</v>
       </c>
-      <c r="O35" s="34">
+      <c r="O35">
         <v>16.86</v>
       </c>
     </row>
     <row r="36" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I36" s="34">
+      <c r="I36">
         <v>7</v>
       </c>
-      <c r="J36" s="34">
+      <c r="J36">
         <v>13.529040925027498</v>
       </c>
-      <c r="K36" s="34">
+      <c r="K36">
         <v>0.85095907497250245</v>
       </c>
-      <c r="L36" s="34">
+      <c r="L36">
         <v>0.5712279323190349</v>
       </c>
-      <c r="N36" s="34">
+      <c r="N36">
         <v>26</v>
       </c>
-      <c r="O36" s="34">
+      <c r="O36">
         <v>17.079999999999998</v>
       </c>
     </row>
     <row r="37" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I37" s="34">
+      <c r="I37">
         <v>8</v>
       </c>
-      <c r="J37" s="34">
+      <c r="J37">
         <v>10.836530460267733</v>
       </c>
-      <c r="K37" s="34">
+      <c r="K37">
         <v>-1.2365304602677334</v>
       </c>
-      <c r="L37" s="34">
+      <c r="L37">
         <v>-0.83005253582972405</v>
       </c>
-      <c r="N37" s="34">
+      <c r="N37">
         <v>30</v>
       </c>
-      <c r="O37" s="34">
+      <c r="O37">
         <v>17.89</v>
       </c>
     </row>
     <row r="38" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I38" s="34">
+      <c r="I38">
         <v>9</v>
       </c>
-      <c r="J38" s="34">
+      <c r="J38">
         <v>26.264546124278478</v>
       </c>
-      <c r="K38" s="34">
+      <c r="K38">
         <v>-1.9145461242784769</v>
       </c>
-      <c r="L38" s="34">
+      <c r="L38">
         <v>-1.2851878028756623</v>
       </c>
-      <c r="N38" s="34">
+      <c r="N38">
         <v>34</v>
       </c>
-      <c r="O38" s="34">
+      <c r="O38">
         <v>21.15</v>
       </c>
     </row>
     <row r="39" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I39" s="34">
+      <c r="I39">
         <v>10</v>
       </c>
-      <c r="J39" s="34">
+      <c r="J39">
         <v>27.596122303133125</v>
       </c>
-      <c r="K39" s="34">
+      <c r="K39">
         <v>-9.6122303133125087E-2</v>
       </c>
-      <c r="L39" s="34">
+      <c r="L39">
         <v>-6.4524541876767455E-2</v>
       </c>
-      <c r="N39" s="34">
+      <c r="N39">
         <v>38</v>
       </c>
-      <c r="O39" s="34">
+      <c r="O39">
         <v>21.65</v>
       </c>
     </row>
     <row r="40" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I40" s="34">
+      <c r="I40">
         <v>11</v>
       </c>
-      <c r="J40" s="34">
+      <c r="J40">
         <v>18.338151586894092</v>
       </c>
-      <c r="K40" s="34">
+      <c r="K40">
         <v>-1.258151586894094</v>
       </c>
-      <c r="L40" s="34">
+      <c r="L40">
         <v>-0.84456626724222827</v>
       </c>
-      <c r="N40" s="34">
+      <c r="N40">
         <v>42</v>
       </c>
-      <c r="O40" s="34">
+      <c r="O40">
         <v>22.13</v>
       </c>
     </row>
     <row r="41" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I41" s="34">
+      <c r="I41">
         <v>12</v>
       </c>
-      <c r="J41" s="34">
+      <c r="J41">
         <v>36.860601158947709</v>
       </c>
-      <c r="K41" s="34">
+      <c r="K41">
         <v>0.13939884105229083</v>
       </c>
-      <c r="L41" s="34">
+      <c r="L41">
         <v>9.3575019156524039E-2</v>
       </c>
-      <c r="N41" s="34">
+      <c r="N41">
         <v>46</v>
       </c>
-      <c r="O41" s="34">
+      <c r="O41">
         <v>24.35</v>
       </c>
     </row>
     <row r="42" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I42" s="34">
+      <c r="I42">
         <v>13</v>
       </c>
-      <c r="J42" s="34">
+      <c r="J42">
         <v>40.786892802764356</v>
       </c>
-      <c r="K42" s="34">
+      <c r="K42">
         <v>1.1631071972356466</v>
       </c>
-      <c r="L42" s="34">
+      <c r="L42">
         <v>0.78076530221359408</v>
       </c>
-      <c r="N42" s="34">
+      <c r="N42">
         <v>50</v>
       </c>
-      <c r="O42" s="34">
+      <c r="O42">
         <v>24.45</v>
       </c>
     </row>
     <row r="43" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I43" s="34">
+      <c r="I43">
         <v>14</v>
       </c>
-      <c r="J43" s="34">
+      <c r="J43">
         <v>13.526098297255755</v>
       </c>
-      <c r="K43" s="34">
+      <c r="K43">
         <v>-1.8660982972557552</v>
       </c>
-      <c r="L43" s="34">
+      <c r="L43">
         <v>-1.2526659661981066</v>
       </c>
-      <c r="N43" s="34">
+      <c r="N43">
         <v>54</v>
       </c>
-      <c r="O43" s="34">
+      <c r="O43">
         <v>25.02</v>
       </c>
     </row>
     <row r="44" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I44" s="34">
+      <c r="I44">
         <v>15</v>
       </c>
-      <c r="J44" s="34">
+      <c r="J44">
         <v>17.03850359318837</v>
       </c>
-      <c r="K44" s="34">
+      <c r="K44">
         <v>4.6114964068116286</v>
       </c>
-      <c r="L44" s="34">
+      <c r="L44">
         <v>3.0955843057961236</v>
       </c>
-      <c r="N44" s="34">
+      <c r="N44">
         <v>58</v>
       </c>
-      <c r="O44" s="34">
+      <c r="O44">
         <v>27.5</v>
       </c>
     </row>
     <row r="45" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I45" s="34">
+      <c r="I45">
         <v>16</v>
       </c>
-      <c r="J45" s="34">
+      <c r="J45">
         <v>18.324650787956152</v>
       </c>
-      <c r="K45" s="34">
+      <c r="K45">
         <v>-0.43465078795615142</v>
       </c>
-      <c r="L45" s="34">
+      <c r="L45">
         <v>-0.29177040140626576</v>
       </c>
-      <c r="N45" s="34">
+      <c r="N45">
         <v>62</v>
       </c>
-      <c r="O45" s="34">
+      <c r="O45">
         <v>31.75</v>
       </c>
     </row>
     <row r="46" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I46" s="34">
+      <c r="I46">
         <v>17</v>
       </c>
-      <c r="J46" s="34">
+      <c r="J46">
         <v>68.49681891852228</v>
       </c>
-      <c r="K46" s="34">
+      <c r="K46">
         <v>0.50318108147772023</v>
       </c>
-      <c r="L46" s="34">
+      <c r="L46">
         <v>0.3377731047334584</v>
       </c>
-      <c r="N46" s="34">
+      <c r="N46">
         <v>66</v>
       </c>
-      <c r="O46" s="34">
+      <c r="O46">
         <v>34.93</v>
       </c>
     </row>
     <row r="47" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I47" s="34">
+      <c r="I47">
         <v>18</v>
       </c>
-      <c r="J47" s="34">
+      <c r="J47">
         <v>9.7186103667495676</v>
       </c>
-      <c r="K47" s="34">
+      <c r="K47">
         <v>0.58138963325043314</v>
       </c>
-      <c r="L47" s="34">
+      <c r="L47">
         <v>0.39027258518172392</v>
       </c>
-      <c r="N47" s="34">
+      <c r="N47">
         <v>70</v>
       </c>
-      <c r="O47" s="34">
+      <c r="O47">
         <v>35</v>
       </c>
     </row>
     <row r="48" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I48" s="34">
+      <c r="I48">
         <v>19</v>
       </c>
-      <c r="J48" s="34">
+      <c r="J48">
         <v>34.98172370790811</v>
       </c>
-      <c r="K48" s="34">
+      <c r="K48">
         <v>-5.1723707908109873E-2</v>
       </c>
-      <c r="L48" s="34">
+      <c r="L48">
         <v>-3.4720855078933209E-2</v>
       </c>
-      <c r="N48" s="34">
+      <c r="N48">
         <v>74</v>
       </c>
-      <c r="O48" s="34">
+      <c r="O48">
         <v>37</v>
       </c>
     </row>
     <row r="49" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I49" s="34">
+      <c r="I49">
         <v>20</v>
       </c>
-      <c r="J49" s="34">
+      <c r="J49">
         <v>45.366981920217633</v>
       </c>
-      <c r="K49" s="34">
+      <c r="K49">
         <v>1.2230180797823706</v>
       </c>
-      <c r="L49" s="34">
+      <c r="L49">
         <v>0.82098200659703291</v>
       </c>
-      <c r="N49" s="34">
+      <c r="N49">
         <v>78</v>
       </c>
-      <c r="O49" s="34">
+      <c r="O49">
         <v>41.95</v>
       </c>
     </row>
     <row r="50" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I50" s="34">
+      <c r="I50">
         <v>21</v>
       </c>
-      <c r="J50" s="34">
+      <c r="J50">
         <v>46.351562819915173</v>
       </c>
-      <c r="K50" s="34">
+      <c r="K50">
         <v>-1.4715628199151709</v>
       </c>
-      <c r="L50" s="34">
+      <c r="L50">
         <v>-0.98782398780443603</v>
       </c>
-      <c r="N50" s="34">
+      <c r="N50">
         <v>82</v>
       </c>
-      <c r="O50" s="34">
+      <c r="O50">
         <v>44.88</v>
       </c>
     </row>
     <row r="51" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I51" s="34">
+      <c r="I51">
         <v>22</v>
       </c>
-      <c r="J51" s="34">
+      <c r="J51">
         <v>53.49173655663256</v>
       </c>
-      <c r="K51" s="34">
+      <c r="K51">
         <v>0.62826344336743745</v>
       </c>
-      <c r="L51" s="34">
+      <c r="L51">
         <v>0.42173782295936518</v>
       </c>
-      <c r="N51" s="34">
+      <c r="N51">
         <v>86</v>
       </c>
-      <c r="O51" s="34">
+      <c r="O51">
         <v>46.59</v>
       </c>
     </row>
     <row r="52" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I52" s="34">
+      <c r="I52">
         <v>23</v>
       </c>
-      <c r="J52" s="34">
+      <c r="J52">
         <v>57.803894748092425</v>
       </c>
-      <c r="K52" s="34">
+      <c r="K52">
         <v>-1.1738947480924224</v>
       </c>
-      <c r="L52" s="34">
+      <c r="L52">
         <v>-0.78800672022291685</v>
       </c>
-      <c r="N52" s="34">
+      <c r="N52">
         <v>90</v>
       </c>
-      <c r="O52" s="34">
+      <c r="O52">
         <v>54.12</v>
       </c>
     </row>
     <row r="53" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I53" s="34">
+      <c r="I53">
         <v>24</v>
       </c>
-      <c r="J53" s="34">
+      <c r="J53">
         <v>19.654292705110532</v>
       </c>
-      <c r="K53" s="34">
+      <c r="K53">
         <v>2.4757072948894674</v>
       </c>
-      <c r="L53" s="34">
+      <c r="L53">
         <v>1.6618815177834014</v>
       </c>
-      <c r="N53" s="34">
+      <c r="N53">
         <v>94</v>
       </c>
-      <c r="O53" s="34">
+      <c r="O53">
         <v>56.63</v>
       </c>
     </row>
     <row r="54" spans="9:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="I54" s="35">
+      <c r="I54" s="33">
         <v>25</v>
       </c>
-      <c r="J54" s="35">
+      <c r="J54" s="33">
         <v>20.813026194568032</v>
       </c>
-      <c r="K54" s="35">
+      <c r="K54" s="33">
         <v>0.33697380543196687</v>
       </c>
-      <c r="L54" s="35">
+      <c r="L54" s="33">
         <v>0.22620224142835449</v>
       </c>
-      <c r="N54" s="35">
+      <c r="N54" s="33">
         <v>98</v>
       </c>
-      <c r="O54" s="35">
+      <c r="O54" s="33">
         <v>69</v>
       </c>
-    </row>
-    <row r="55" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I55" s="34"/>
-      <c r="J55" s="34"/>
-      <c r="K55" s="34"/>
-      <c r="L55" s="34"/>
-      <c r="N55" s="34"/>
-      <c r="O55" s="34"/>
-    </row>
-    <row r="56" spans="9:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I56" s="34"/>
-      <c r="J56" s="34"/>
-      <c r="K56" s="34"/>
-      <c r="L56" s="34"/>
-      <c r="N56" s="34"/>
-      <c r="O56" s="34"/>
     </row>
     <row r="57" spans="9:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="I57" s="35"/>
-      <c r="J57" s="35"/>
-      <c r="K57" s="35"/>
-      <c r="L57" s="35"/>
-      <c r="N57" s="35"/>
-      <c r="O57" s="35"/>
+      <c r="I57" s="33"/>
+      <c r="J57" s="33"/>
+      <c r="K57" s="33"/>
+      <c r="L57" s="33"/>
+      <c r="N57" s="33"/>
+      <c r="O57" s="33"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="O30:O54">

</xml_diff>